<commit_message>
docs: refine project proposal, HU and MER documentation with architectural improvements
</commit_message>
<xml_diff>
--- a/docs/INFORME DE PROYECTO DE AULA.xlsx
+++ b/docs/INFORME DE PROYECTO DE AULA.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marianapereiraospina/Desktop/ARQUITECTURA DE SOFTWARE/Corte 2/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marianapereiraospina/Desktop/ARQUITECTURA DE SOFTWARE/Corte 3/Home-Health/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AAA561F9-3B29-7B40-B5AE-31ED65DD63A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97762D26-21D0-6D4B-B305-44E685A79D47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="18380" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="16660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="INFORME" sheetId="1" r:id="rId1"/>
@@ -916,12 +916,6 @@
     <t>Ingeniería de software</t>
   </si>
   <si>
-    <t xml:space="preserve"> 12/03/2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 27/03/2026</t>
-  </si>
-  <si>
     <t>Facultad de Ingeniería</t>
   </si>
   <si>
@@ -948,11 +942,6 @@
 Los beneficiarios directos del proyecto serán los estudiantes participantes, quienes fortalecerán sus competencias en desarrollo de software y arquitectura de sistemas. De manera indirecta, el proyecto puede servir como referencia para el desarrollo de soluciones tecnológicas similares orientadas a la gestión de inventarios en establecimientos comerciales del sector farmacéutico.</t>
   </si>
   <si>
-    <t>Desarrollo de software
-Sitio web
-Presentaciones educativas (diapositivas)</t>
-  </si>
-  <si>
     <t>Anexo 1: Capturas del sistema web desarrollado
 Anexo 2: Diagramas de arquitectura y modelo de base de datos
 Anexo 3: Evidencias del proceso de desarrollo del proyecto</t>
@@ -961,13 +950,6 @@
     <t>Consejo Nacional de Política Económica y Social (CONPES). (2012). Política farmacéutica nacional. Departamento Nacional de Planeación. https://www.minsalud.gov.co/salud/MT/Paginas/medicamentos-conpes-155.aspx                                                                                                                                                                                  Ministerio de la Protección Social. (2005). Decreto 2200 de 2005: Por el cual se reglamenta el servicio farmacéutico. https://www.funcionpublica.gov.co/eva/gestornormativo/norma.php?i=16944                                                                                                                                                                                                                                                                                                            Departamento Administrativo Nacional de Estadística (DANE). (2026). Encuesta mensual de comercio (EMC). https://www.dane.gov.co/index.php/estadisticas-por-tema/comercio-interno/encuesta-mensual-de-comercio-emc</t>
   </si>
   <si>
-    <t>Como resultado del proyecto se espera el desarrollo de un sistema web funcional que permita visualizar productos farmacéuticos organizados por categorías, registrar solicitudes de pedidos y gestionar el inventario mediante un módulo administrativo, con el fin de simular procesos de gestión de inventario en establecimientos farmacéuticos.
-Entre las evidencias del proyecto se encuentran el sistema web desarrollado, la documentación de la arquitectura del software, el modelo de base de datos, el código fuente del sistema y las pruebas realizadas durante el proceso de implementación.
-El proyecto será desarrollado por los estudiantes participantes del curso, quienes llevarán a cabo actividades relacionadas con el análisis del problema, el diseño del sistema, la implementación del software y la realización de pruebas. Se espera alcanzar el cumplimiento de las actividades definidas dentro del proyecto y la implementación del sistema propuesto en un entorno de simulación académica.
-Desde el punto de vista académico, el proyecto contribuirá al fortalecimiento de competencias en desarrollo de software, arquitectura de software, diseño de bases de datos y trabajo colaborativo. Asimismo, permitirá aplicar conocimientos teóricos en un ejercicio práctico relacionado con la simulación de procesos de gestión de información en establecimientos farmacéuticos.
-Los resultados del proyecto podrán ser socializados mediante la presentación del sistema desarrollado y la documentación del proceso de desarrollo dentro del contexto académico.</t>
-  </si>
-  <si>
     <t>CORHUILA</t>
   </si>
   <si>
@@ -989,22 +971,46 @@
     <t>Desarrollo de un sistema web para la gestión de inventario y pedidos en farmacias</t>
   </si>
   <si>
-    <t>Desarrollar un sistema de información web para la gestión, seguimiento y generación automatizada de informes de proyectos de aula (Formato FO-IV-159), mediante una arquitectura de software por capas y un diseño centrado en el usuario, con el fin de optimizar los tiempos de reporte y asegurar la integridad de la información académica en la institución.</t>
-  </si>
-  <si>
-    <t>1. Analizar los requisitos funcionales y no funcionales basados en el formato FO-IV-159 y las necesidades de los roles (docentes, estudiantes, coordinadores) para definir el alcance técnico del MVP.
-2. Diseñar la arquitectura de software y el modelo de datos relacional que soporte la jerarquía de facultades, programas, proyectos y productos detallados en las listas institucionales.
-3. Construir los módulos de captura de datos (formularios dinámicos) y gestión de talento humano utilizando un stack tecnológico moderno que garantice la escalabilidad del sistema.
-4. Implementar un motor de generación de documentos que exporte automáticamente la información procesada al formato oficial requerido por la oficina de investigaciones.
-5. Validar la funcionalidad y usabilidad del sistema mediante pruebas de caja negra y retroalimentación de usuarios finales para asegurar el cumplimiento del cronograma de 2.5 meses.</t>
+    <t>Desarrollar un sistema web para la gestión de inventario y solicitudes de pedidos en farmacias, mediante una arquitectura cliente-servidor, que permita el control de stock, la organización de medicamentos por categorías y el seguimiento de productos próximos a vencer.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 25/05/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 11/04/2026</t>
+  </si>
+  <si>
+    <t>Sistema web funcional
+Modelo de base de datos
+Documentación técnica
+Diagramas de arquitectura
+Código fuente</t>
+  </si>
+  <si>
+    <t>1. Analizar los requisitos funcionales y no funcionales del sistema de gestión farmacéutica para definir el alcance técnico y operativo de la plataforma web.
+2. Diseñar la arquitectura de software y el modelo de base de datos relacional que permitan gestionar usuarios, productos, inventario, pedidos y control de vencimientos.
+3. Desarrollar los módulos del sistema utilizando tecnologías web modernas que permitan la administración de inventario, el registro de pedidos y la autenticación de usuarios mediante servicios REST.
+4. Implementar funcionalidades de monitoreo y notificación para el control de stock y productos próximos a vencer, facilitando la gestión operativa de farmacias y droguerías.
+5. Validar la funcionalidad y usabilidad del sistema mediante pruebas de software y revisión de los requerimientos definidos, asegurando el correcto funcionamiento de la plataforma dentro del cronograma establecido.</t>
   </si>
   <si>
     <t>Metodología Principal: Aprendizaje Basado en Proyectos (ABP)
-Justificación: El desarrollo del software es en sí mismo el "proyecto de aula". Se centra en resolver una problemática real (la ineficiencia de llenar informes en Excel/Word manualmente) mediante la construcción de un artefacto tecnológico.
-Aplicación: El equipo de 2 desarrolladores asume roles de arquitecto y programador, enfrentando desafíos técnicos reales (manejo de estados, persistencia de datos, generación de PDF) cuya resolución constituye el aprendizaje principal.
+Justificación:
+El desarrollo del sistema web Home-Health constituye el proyecto de aula, orientado a resolver problemáticas relacionadas con la gestión de inventario y pedidos en farmacias y droguerías mediante la construcción de una solución tecnológica funcional.
+Aplicación:
+El equipo de 3 desarrolladores asume roles relacionados con análisis, diseño, desarrollo backend, frontend y arquitectura de software, enfrentando desafíos técnicos reales como autenticación mediante JWT, gestión de estados de pedidos, control de inventario y despliegue de servicios en contenedores Docker y entornos cloud.
 Metodología Complementaria: Design Thinking
-Justificación: Es vital para que la interfaz sea fácil de usar para los docentes que no son del área de sistemas.
-Aplicación: Se utiliza en la fase inicial para "Empatizar" con los usuarios que hoy sufren llenando el Excel, "Definir" los campos críticos y "Prototipar" las pantallas antes de programar a fondo, asegurando que el producto final sea realmente útil.</t>
+Justificación:
+La metodología permite diseñar una plataforma centrada en la experiencia del usuario, facilitando la interacción tanto para administradores como para clientes del sistema.
+Aplicación:
+Se aplica durante las etapas iniciales del proyecto para identificar necesidades del entorno farmacéutico, definir funcionalidades prioritarias y prototipar interfaces que faciliten la navegación, gestión de productos y seguimiento de pedidos antes de iniciar el desarrollo completo del sistema.</t>
+  </si>
+  <si>
+    <t>Como resultado del proyecto se espera el desarrollo de un sistema web funcional denominado Home-Health, orientado a la gestión de inventario y solicitudes de pedidos en farmacias y droguerías. La plataforma permitirá administrar productos farmacéuticos organizados por categorías, controlar existencias, monitorear fechas de vencimiento y registrar solicitudes de pedidos mediante diferentes niveles de acceso para administradores y clientes.
+Entre las evidencias del proyecto se encuentran el sistema web desarrollado, la documentación de arquitectura de software, el modelo entidad-relación de la base de datos, la documentación de los servicios REST, los diagramas arquitectónicos, el código fuente del sistema y las pruebas realizadas durante el proceso de implementación.
+El proyecto será desarrollado por los estudiantes participantes del curso, quienes ejecutarán actividades relacionadas con el análisis de requisitos, diseño de arquitectura, modelado de base de datos, implementación de servicios backend, desarrollo frontend y pruebas funcionales del sistema.
+Desde el punto de vista académico, el proyecto contribuirá al fortalecimiento de competencias en desarrollo web, arquitectura de software, diseño de APIs REST, contenedorización con Docker, despliegue en servicios cloud y trabajo colaborativo en equipos de desarrollo.
+Finalmente, los resultados obtenidos serán socializados mediante la presentación funcional del sistema Home-Health y la documentación técnica y académica generada durante el desarrollo del proyecto.</t>
   </si>
 </sst>
 </file>
@@ -2796,7 +2802,7 @@
       </c>
       <c r="C7" s="58"/>
       <c r="D7" s="81" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="E7" s="82"/>
       <c r="F7" s="83"/>
@@ -2838,7 +2844,7 @@
       </c>
       <c r="C10" s="58"/>
       <c r="D10" s="81" t="s">
-        <v>281</v>
+        <v>297</v>
       </c>
       <c r="E10" s="82"/>
       <c r="F10" s="83"/>
@@ -2852,7 +2858,7 @@
       </c>
       <c r="C11" s="58"/>
       <c r="D11" s="81" t="s">
-        <v>282</v>
+        <v>296</v>
       </c>
       <c r="E11" s="82"/>
       <c r="F11" s="83"/>
@@ -2866,7 +2872,7 @@
       </c>
       <c r="C12" s="58"/>
       <c r="D12" s="87" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="E12" s="88"/>
       <c r="F12" s="89"/>
@@ -2880,7 +2886,7 @@
       </c>
       <c r="C13" s="58"/>
       <c r="D13" s="84" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="E13" s="85"/>
       <c r="F13" s="86"/>
@@ -2933,7 +2939,7 @@
       </c>
       <c r="C17" s="58"/>
       <c r="D17" s="81" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="E17" s="82"/>
       <c r="F17" s="83"/>
@@ -2947,7 +2953,7 @@
       </c>
       <c r="C18" s="58"/>
       <c r="D18" s="61" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="E18" s="62"/>
       <c r="F18" s="63"/>
@@ -2961,7 +2967,7 @@
       </c>
       <c r="C19" s="58"/>
       <c r="D19" s="81" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="E19" s="82"/>
       <c r="F19" s="83"/>
@@ -2985,12 +2991,12 @@
       </c>
       <c r="C21" s="58"/>
       <c r="D21" s="81" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
       <c r="E21" s="82"/>
       <c r="F21" s="83"/>
     </row>
-    <row r="22" spans="1:7" ht="202" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:7" ht="110" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="50">
         <v>16</v>
       </c>
@@ -2999,12 +3005,12 @@
       </c>
       <c r="C22" s="58"/>
       <c r="D22" s="81" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="E22" s="82"/>
       <c r="F22" s="83"/>
     </row>
-    <row r="23" spans="1:7" ht="280" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:7" ht="284" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="50">
         <v>17</v>
       </c>
@@ -3013,7 +3019,7 @@
       </c>
       <c r="C23" s="58"/>
       <c r="D23" s="81" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="E23" s="82"/>
       <c r="F23" s="83"/>
@@ -3038,13 +3044,13 @@
       </c>
       <c r="C25" s="58"/>
       <c r="D25" s="90" t="s">
-        <v>291</v>
+        <v>301</v>
       </c>
       <c r="E25" s="91"/>
       <c r="F25" s="92"/>
       <c r="G25" s="43"/>
     </row>
-    <row r="26" spans="1:7" ht="62" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:7" ht="111" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="50">
         <v>19</v>
       </c>
@@ -3053,7 +3059,7 @@
       </c>
       <c r="C26" s="60"/>
       <c r="D26" s="90" t="s">
-        <v>288</v>
+        <v>298</v>
       </c>
       <c r="E26" s="91"/>
       <c r="F26" s="92"/>
@@ -3078,7 +3084,7 @@
       </c>
       <c r="C28" s="58"/>
       <c r="D28" s="61" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="E28" s="62"/>
       <c r="F28" s="63"/>
@@ -3102,7 +3108,7 @@
       </c>
       <c r="C30" s="58"/>
       <c r="D30" s="61" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="E30" s="62"/>
       <c r="F30" s="63"/>
@@ -5987,7 +5993,11 @@
     <mergeCell ref="D30:F30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
-  <pageSetup paperSize="9" scale="38" orientation="landscape" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="37" orientation="landscape" r:id="rId1"/>
+  <rowBreaks count="2" manualBreakCount="2">
+    <brk id="18" max="5" man="1"/>
+    <brk id="27" max="5" man="1"/>
+  </rowBreaks>
   <drawing r:id="rId2"/>
 </worksheet>
 </file>
@@ -6046,19 +6056,19 @@
     </row>
     <row r="4" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>293</v>
+        <v>289</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>294</v>
+        <v>290</v>
       </c>
       <c r="D4" s="6">
         <v>7</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>295</v>
+        <v>291</v>
       </c>
       <c r="F4" s="6">
         <v>1077225054</v>
@@ -6066,19 +6076,19 @@
     </row>
     <row r="5" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>293</v>
+        <v>289</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>294</v>
+        <v>290</v>
       </c>
       <c r="D5" s="6">
         <v>6</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>296</v>
+        <v>292</v>
       </c>
       <c r="F5" s="6">
         <v>1077847063</v>
@@ -6086,19 +6096,19 @@
     </row>
     <row r="6" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="5" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>293</v>
+        <v>289</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>294</v>
+        <v>290</v>
       </c>
       <c r="D6" s="6">
         <v>6</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>297</v>
+        <v>293</v>
       </c>
       <c r="F6" s="6">
         <v>1077723138</v>

</xml_diff>

<commit_message>
docs: update deployment architecture to AWS EC2
</commit_message>
<xml_diff>
--- a/docs/INFORME DE PROYECTO DE AULA.xlsx
+++ b/docs/INFORME DE PROYECTO DE AULA.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marianapereiraospina/Desktop/ARQUITECTURA DE SOFTWARE/Corte 3/Home-Health/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97762D26-21D0-6D4B-B305-44E685A79D47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC511DDF-0CD7-4E4A-9B35-3FC3C1CA4DC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="16660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="16660" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="INFORME" sheetId="1" r:id="rId1"/>
@@ -1704,27 +1704,14 @@
     <xf numFmtId="0" fontId="6" fillId="7" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
@@ -1733,6 +1720,49 @@
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1780,47 +1810,17 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2673,27 +2673,27 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="64"/>
-      <c r="B1" s="65"/>
-      <c r="C1" s="76" t="s">
+      <c r="A1" s="74"/>
+      <c r="B1" s="75"/>
+      <c r="C1" s="86" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="77"/>
-      <c r="E1" s="77"/>
-      <c r="F1" s="78"/>
+      <c r="D1" s="87"/>
+      <c r="E1" s="87"/>
+      <c r="F1" s="88"/>
       <c r="G1" s="32"/>
       <c r="H1" s="32"/>
       <c r="I1" s="32"/>
     </row>
     <row r="2" spans="1:20" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="66"/>
-      <c r="B2" s="67"/>
-      <c r="C2" s="70" t="s">
+      <c r="A2" s="76"/>
+      <c r="B2" s="77"/>
+      <c r="C2" s="80" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="71"/>
-      <c r="E2" s="71"/>
-      <c r="F2" s="72"/>
+      <c r="D2" s="81"/>
+      <c r="E2" s="81"/>
+      <c r="F2" s="82"/>
       <c r="G2" s="32"/>
       <c r="H2" s="32"/>
       <c r="I2" s="32"/>
@@ -2710,12 +2710,12 @@
       <c r="T2" s="32"/>
     </row>
     <row r="3" spans="1:20" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="66"/>
-      <c r="B3" s="67"/>
-      <c r="C3" s="73"/>
-      <c r="D3" s="74"/>
-      <c r="E3" s="74"/>
-      <c r="F3" s="75"/>
+      <c r="A3" s="76"/>
+      <c r="B3" s="77"/>
+      <c r="C3" s="83"/>
+      <c r="D3" s="84"/>
+      <c r="E3" s="84"/>
+      <c r="F3" s="85"/>
       <c r="G3" s="32"/>
       <c r="H3" s="32"/>
       <c r="I3" s="32"/>
@@ -2732,8 +2732,8 @@
       <c r="T3" s="32"/>
     </row>
     <row r="4" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="68"/>
-      <c r="B4" s="69"/>
+      <c r="A4" s="78"/>
+      <c r="B4" s="79"/>
       <c r="C4" s="42" t="s">
         <v>2</v>
       </c>
@@ -2762,12 +2762,12 @@
       <c r="T4" s="32"/>
     </row>
     <row r="5" spans="1:20" ht="1.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="79"/>
-      <c r="B5" s="79"/>
-      <c r="C5" s="54"/>
-      <c r="D5" s="54"/>
-      <c r="E5" s="54"/>
-      <c r="F5" s="54"/>
+      <c r="A5" s="69"/>
+      <c r="B5" s="69"/>
+      <c r="C5" s="66"/>
+      <c r="D5" s="66"/>
+      <c r="E5" s="66"/>
+      <c r="F5" s="66"/>
       <c r="G5" s="32"/>
       <c r="H5" s="32"/>
       <c r="I5" s="32"/>
@@ -2784,352 +2784,352 @@
       <c r="T5" s="32"/>
     </row>
     <row r="6" spans="1:20" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="80" t="s">
+      <c r="A6" s="70" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="80"/>
-      <c r="C6" s="54"/>
-      <c r="D6" s="54"/>
-      <c r="E6" s="54"/>
-      <c r="F6" s="54"/>
+      <c r="B6" s="70"/>
+      <c r="C6" s="66"/>
+      <c r="D6" s="66"/>
+      <c r="E6" s="66"/>
+      <c r="F6" s="66"/>
     </row>
     <row r="7" spans="1:20" ht="71.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="50">
         <v>1</v>
       </c>
-      <c r="B7" s="57" t="s">
+      <c r="B7" s="67" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="58"/>
-      <c r="D7" s="81" t="s">
+      <c r="C7" s="68"/>
+      <c r="D7" s="62" t="s">
         <v>294</v>
       </c>
-      <c r="E7" s="82"/>
-      <c r="F7" s="83"/>
+      <c r="E7" s="63"/>
+      <c r="F7" s="64"/>
     </row>
     <row r="8" spans="1:20" ht="171" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="50">
         <v>2</v>
       </c>
-      <c r="B8" s="57" t="s">
+      <c r="B8" s="67" t="s">
         <v>8</v>
       </c>
-      <c r="C8" s="58"/>
-      <c r="D8" s="81" t="s">
+      <c r="C8" s="68"/>
+      <c r="D8" s="62" t="s">
         <v>279</v>
       </c>
-      <c r="E8" s="82"/>
-      <c r="F8" s="83"/>
+      <c r="E8" s="63"/>
+      <c r="F8" s="64"/>
     </row>
     <row r="9" spans="1:20" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="50">
         <v>3</v>
       </c>
-      <c r="B9" s="57" t="s">
+      <c r="B9" s="67" t="s">
         <v>9</v>
       </c>
-      <c r="C9" s="58"/>
-      <c r="D9" s="84" t="s">
+      <c r="C9" s="68"/>
+      <c r="D9" s="71" t="s">
         <v>280</v>
       </c>
-      <c r="E9" s="85"/>
-      <c r="F9" s="86"/>
+      <c r="E9" s="72"/>
+      <c r="F9" s="73"/>
     </row>
     <row r="10" spans="1:20" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="50">
         <v>5</v>
       </c>
-      <c r="B10" s="57" t="s">
+      <c r="B10" s="67" t="s">
         <v>10</v>
       </c>
-      <c r="C10" s="58"/>
-      <c r="D10" s="81" t="s">
+      <c r="C10" s="68"/>
+      <c r="D10" s="62" t="s">
         <v>297</v>
       </c>
-      <c r="E10" s="82"/>
-      <c r="F10" s="83"/>
+      <c r="E10" s="63"/>
+      <c r="F10" s="64"/>
     </row>
     <row r="11" spans="1:20" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="50">
         <v>6</v>
       </c>
-      <c r="B11" s="57" t="s">
+      <c r="B11" s="67" t="s">
         <v>11</v>
       </c>
-      <c r="C11" s="58"/>
-      <c r="D11" s="81" t="s">
+      <c r="C11" s="68"/>
+      <c r="D11" s="62" t="s">
         <v>296</v>
       </c>
-      <c r="E11" s="82"/>
-      <c r="F11" s="83"/>
+      <c r="E11" s="63"/>
+      <c r="F11" s="64"/>
     </row>
     <row r="12" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="50">
         <v>8</v>
       </c>
-      <c r="B12" s="57" t="s">
+      <c r="B12" s="67" t="s">
         <v>12</v>
       </c>
-      <c r="C12" s="58"/>
-      <c r="D12" s="87" t="s">
+      <c r="C12" s="68"/>
+      <c r="D12" s="53" t="s">
         <v>281</v>
       </c>
-      <c r="E12" s="88"/>
-      <c r="F12" s="89"/>
+      <c r="E12" s="54"/>
+      <c r="F12" s="55"/>
     </row>
     <row r="13" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A13" s="50">
         <v>9</v>
       </c>
-      <c r="B13" s="57" t="s">
+      <c r="B13" s="67" t="s">
         <v>13</v>
       </c>
-      <c r="C13" s="58"/>
-      <c r="D13" s="84" t="s">
+      <c r="C13" s="68"/>
+      <c r="D13" s="71" t="s">
         <v>282</v>
       </c>
-      <c r="E13" s="85"/>
-      <c r="F13" s="86"/>
+      <c r="E13" s="72"/>
+      <c r="F13" s="73"/>
     </row>
     <row r="14" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="50">
         <v>10</v>
       </c>
-      <c r="B14" s="57" t="s">
+      <c r="B14" s="67" t="s">
         <v>14</v>
       </c>
-      <c r="C14" s="58"/>
-      <c r="D14" s="87">
+      <c r="C14" s="68"/>
+      <c r="D14" s="53">
         <v>6</v>
       </c>
-      <c r="E14" s="88"/>
-      <c r="F14" s="89"/>
+      <c r="E14" s="54"/>
+      <c r="F14" s="55"/>
     </row>
     <row r="15" spans="1:20" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="50">
         <v>11</v>
       </c>
-      <c r="B15" s="57" t="s">
+      <c r="B15" s="67" t="s">
         <v>15</v>
       </c>
-      <c r="C15" s="58"/>
-      <c r="D15" s="87">
+      <c r="C15" s="68"/>
+      <c r="D15" s="53">
         <v>3</v>
       </c>
-      <c r="E15" s="88"/>
-      <c r="F15" s="89"/>
+      <c r="E15" s="54"/>
+      <c r="F15" s="55"/>
       <c r="G15" s="44"/>
     </row>
     <row r="16" spans="1:20" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="56" t="s">
+      <c r="A16" s="65" t="s">
         <v>16</v>
       </c>
-      <c r="B16" s="56"/>
-      <c r="C16" s="54"/>
-      <c r="D16" s="54"/>
-      <c r="E16" s="54"/>
-      <c r="F16" s="54"/>
+      <c r="B16" s="65"/>
+      <c r="C16" s="66"/>
+      <c r="D16" s="66"/>
+      <c r="E16" s="66"/>
+      <c r="F16" s="66"/>
     </row>
     <row r="17" spans="1:7" ht="409" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="50">
         <v>12</v>
       </c>
-      <c r="B17" s="57" t="s">
+      <c r="B17" s="67" t="s">
         <v>17</v>
       </c>
-      <c r="C17" s="58"/>
-      <c r="D17" s="81" t="s">
+      <c r="C17" s="68"/>
+      <c r="D17" s="62" t="s">
         <v>283</v>
       </c>
-      <c r="E17" s="82"/>
-      <c r="F17" s="83"/>
+      <c r="E17" s="63"/>
+      <c r="F17" s="64"/>
     </row>
     <row r="18" spans="1:7" ht="88.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="50">
         <v>13</v>
       </c>
-      <c r="B18" s="57" t="s">
+      <c r="B18" s="67" t="s">
         <v>18</v>
       </c>
-      <c r="C18" s="58"/>
-      <c r="D18" s="61" t="s">
+      <c r="C18" s="68"/>
+      <c r="D18" s="56" t="s">
         <v>284</v>
       </c>
-      <c r="E18" s="62"/>
-      <c r="F18" s="63"/>
+      <c r="E18" s="57"/>
+      <c r="F18" s="58"/>
     </row>
     <row r="19" spans="1:7" ht="409" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="50">
         <v>14</v>
       </c>
-      <c r="B19" s="57" t="s">
+      <c r="B19" s="67" t="s">
         <v>19</v>
       </c>
-      <c r="C19" s="58"/>
-      <c r="D19" s="81" t="s">
+      <c r="C19" s="68"/>
+      <c r="D19" s="62" t="s">
         <v>285</v>
       </c>
-      <c r="E19" s="82"/>
-      <c r="F19" s="83"/>
+      <c r="E19" s="63"/>
+      <c r="F19" s="64"/>
     </row>
     <row r="20" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="56" t="s">
+      <c r="A20" s="65" t="s">
         <v>20</v>
       </c>
-      <c r="B20" s="56"/>
-      <c r="C20" s="54"/>
-      <c r="D20" s="54"/>
-      <c r="E20" s="54"/>
-      <c r="F20" s="54"/>
+      <c r="B20" s="65"/>
+      <c r="C20" s="66"/>
+      <c r="D20" s="66"/>
+      <c r="E20" s="66"/>
+      <c r="F20" s="66"/>
     </row>
     <row r="21" spans="1:7" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="50">
         <v>15</v>
       </c>
-      <c r="B21" s="57" t="s">
+      <c r="B21" s="67" t="s">
         <v>21</v>
       </c>
-      <c r="C21" s="58"/>
-      <c r="D21" s="81" t="s">
+      <c r="C21" s="68"/>
+      <c r="D21" s="62" t="s">
         <v>295</v>
       </c>
-      <c r="E21" s="82"/>
-      <c r="F21" s="83"/>
+      <c r="E21" s="63"/>
+      <c r="F21" s="64"/>
     </row>
     <row r="22" spans="1:7" ht="110" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="50">
         <v>16</v>
       </c>
-      <c r="B22" s="57" t="s">
+      <c r="B22" s="67" t="s">
         <v>22</v>
       </c>
-      <c r="C22" s="58"/>
-      <c r="D22" s="81" t="s">
+      <c r="C22" s="68"/>
+      <c r="D22" s="62" t="s">
         <v>299</v>
       </c>
-      <c r="E22" s="82"/>
-      <c r="F22" s="83"/>
+      <c r="E22" s="63"/>
+      <c r="F22" s="64"/>
     </row>
     <row r="23" spans="1:7" ht="284" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="50">
         <v>17</v>
       </c>
-      <c r="B23" s="57" t="s">
+      <c r="B23" s="67" t="s">
         <v>23</v>
       </c>
-      <c r="C23" s="58"/>
-      <c r="D23" s="81" t="s">
+      <c r="C23" s="68"/>
+      <c r="D23" s="62" t="s">
         <v>300</v>
       </c>
-      <c r="E23" s="82"/>
-      <c r="F23" s="83"/>
+      <c r="E23" s="63"/>
+      <c r="F23" s="64"/>
       <c r="G23" s="43"/>
     </row>
     <row r="24" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="56" t="s">
+      <c r="A24" s="65" t="s">
         <v>24</v>
       </c>
-      <c r="B24" s="56"/>
-      <c r="C24" s="54"/>
-      <c r="D24" s="54"/>
-      <c r="E24" s="54"/>
-      <c r="F24" s="54"/>
+      <c r="B24" s="65"/>
+      <c r="C24" s="66"/>
+      <c r="D24" s="66"/>
+      <c r="E24" s="66"/>
+      <c r="F24" s="66"/>
     </row>
     <row r="25" spans="1:7" ht="267" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="50">
         <v>18</v>
       </c>
-      <c r="B25" s="57" t="s">
+      <c r="B25" s="67" t="s">
         <v>25</v>
       </c>
-      <c r="C25" s="58"/>
-      <c r="D25" s="90" t="s">
+      <c r="C25" s="68"/>
+      <c r="D25" s="59" t="s">
         <v>301</v>
       </c>
-      <c r="E25" s="91"/>
-      <c r="F25" s="92"/>
+      <c r="E25" s="60"/>
+      <c r="F25" s="61"/>
       <c r="G25" s="43"/>
     </row>
     <row r="26" spans="1:7" ht="111" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="50">
         <v>19</v>
       </c>
-      <c r="B26" s="59" t="s">
+      <c r="B26" s="91" t="s">
         <v>26</v>
       </c>
-      <c r="C26" s="60"/>
-      <c r="D26" s="90" t="s">
+      <c r="C26" s="92"/>
+      <c r="D26" s="59" t="s">
         <v>298</v>
       </c>
-      <c r="E26" s="91"/>
-      <c r="F26" s="92"/>
+      <c r="E26" s="60"/>
+      <c r="F26" s="61"/>
       <c r="G26" s="43"/>
     </row>
     <row r="27" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="56" t="s">
+      <c r="A27" s="65" t="s">
         <v>27</v>
       </c>
-      <c r="B27" s="56"/>
-      <c r="C27" s="54"/>
-      <c r="D27" s="54"/>
-      <c r="E27" s="54"/>
-      <c r="F27" s="54"/>
+      <c r="B27" s="65"/>
+      <c r="C27" s="66"/>
+      <c r="D27" s="66"/>
+      <c r="E27" s="66"/>
+      <c r="F27" s="66"/>
     </row>
     <row r="28" spans="1:7" ht="63.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="50">
         <v>20</v>
       </c>
-      <c r="B28" s="57" t="s">
+      <c r="B28" s="67" t="s">
         <v>28</v>
       </c>
-      <c r="C28" s="58"/>
-      <c r="D28" s="61" t="s">
+      <c r="C28" s="68"/>
+      <c r="D28" s="56" t="s">
         <v>286</v>
       </c>
-      <c r="E28" s="62"/>
-      <c r="F28" s="63"/>
+      <c r="E28" s="57"/>
+      <c r="F28" s="58"/>
     </row>
     <row r="29" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="56" t="s">
+      <c r="A29" s="65" t="s">
         <v>29</v>
       </c>
-      <c r="B29" s="56"/>
-      <c r="C29" s="54"/>
-      <c r="D29" s="54"/>
-      <c r="E29" s="54"/>
-      <c r="F29" s="54"/>
+      <c r="B29" s="65"/>
+      <c r="C29" s="66"/>
+      <c r="D29" s="66"/>
+      <c r="E29" s="66"/>
+      <c r="F29" s="66"/>
     </row>
     <row r="30" spans="1:7" ht="127" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="50">
         <v>21</v>
       </c>
-      <c r="B30" s="57" t="s">
+      <c r="B30" s="67" t="s">
         <v>30</v>
       </c>
-      <c r="C30" s="58"/>
-      <c r="D30" s="61" t="s">
+      <c r="C30" s="68"/>
+      <c r="D30" s="56" t="s">
         <v>287</v>
       </c>
-      <c r="E30" s="62"/>
-      <c r="F30" s="63"/>
+      <c r="E30" s="57"/>
+      <c r="F30" s="58"/>
     </row>
     <row r="31" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="53"/>
-      <c r="B31" s="53"/>
-      <c r="C31" s="54"/>
-      <c r="D31" s="54"/>
-      <c r="E31" s="54"/>
-      <c r="F31" s="54"/>
+      <c r="A31" s="89"/>
+      <c r="B31" s="89"/>
+      <c r="C31" s="66"/>
+      <c r="D31" s="66"/>
+      <c r="E31" s="66"/>
+      <c r="F31" s="66"/>
     </row>
     <row r="32" spans="1:7" ht="33" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="55" t="s">
+      <c r="A32" s="90" t="s">
         <v>31</v>
       </c>
-      <c r="B32" s="55"/>
-      <c r="C32" s="54"/>
-      <c r="D32" s="54"/>
-      <c r="E32" s="54"/>
-      <c r="F32" s="54"/>
+      <c r="B32" s="90"/>
+      <c r="C32" s="66"/>
+      <c r="D32" s="66"/>
+      <c r="E32" s="66"/>
+      <c r="F32" s="66"/>
     </row>
     <row r="33" spans="6:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="F33" s="1"/>
@@ -5941,6 +5941,40 @@
     </row>
   </sheetData>
   <mergeCells count="50">
+    <mergeCell ref="A31:F31"/>
+    <mergeCell ref="A32:F32"/>
+    <mergeCell ref="A24:F24"/>
+    <mergeCell ref="A27:F27"/>
+    <mergeCell ref="A29:F29"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="D30:F30"/>
+    <mergeCell ref="A1:B4"/>
+    <mergeCell ref="C2:F3"/>
+    <mergeCell ref="C1:F1"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="A20:F20"/>
+    <mergeCell ref="A5:F5"/>
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="D7:F7"/>
+    <mergeCell ref="D8:F8"/>
+    <mergeCell ref="D9:F9"/>
+    <mergeCell ref="D10:F10"/>
+    <mergeCell ref="D11:F11"/>
+    <mergeCell ref="D12:F12"/>
+    <mergeCell ref="D13:F13"/>
+    <mergeCell ref="D14:F14"/>
     <mergeCell ref="D15:F15"/>
     <mergeCell ref="D28:F28"/>
     <mergeCell ref="D26:F26"/>
@@ -5957,40 +5991,6 @@
     <mergeCell ref="B23:C23"/>
     <mergeCell ref="B22:C22"/>
     <mergeCell ref="B21:C21"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="A20:F20"/>
-    <mergeCell ref="A5:F5"/>
-    <mergeCell ref="A6:F6"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="D7:F7"/>
-    <mergeCell ref="D8:F8"/>
-    <mergeCell ref="D9:F9"/>
-    <mergeCell ref="D10:F10"/>
-    <mergeCell ref="D11:F11"/>
-    <mergeCell ref="D12:F12"/>
-    <mergeCell ref="D13:F13"/>
-    <mergeCell ref="D14:F14"/>
-    <mergeCell ref="A1:B4"/>
-    <mergeCell ref="C2:F3"/>
-    <mergeCell ref="C1:F1"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="A31:F31"/>
-    <mergeCell ref="A32:F32"/>
-    <mergeCell ref="A24:F24"/>
-    <mergeCell ref="A27:F27"/>
-    <mergeCell ref="A29:F29"/>
-    <mergeCell ref="B30:C30"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="B25:C25"/>
-    <mergeCell ref="D30:F30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup paperSize="9" scale="37" orientation="landscape" r:id="rId1"/>
@@ -13225,26 +13225,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="c7b9d0d2-0928-4bc7-b1e7-d815d07dd502" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3b21ab7c-7e7a-493b-a43f-a219844d5b04">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x01010076AC4B3079F3F14986B23BC4E8B1044F" ma:contentTypeVersion="16" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="b5e42e84a51bf8907db879a7bd14d01e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="3b21ab7c-7e7a-493b-a43f-a219844d5b04" xmlns:ns3="c7b9d0d2-0928-4bc7-b1e7-d815d07dd502" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d18fa931cd5ae0925a29b1e6f4a02f35" ns2:_="" ns3:_="">
     <xsd:import namespace="3b21ab7c-7e7a-493b-a43f-a219844d5b04"/>
@@ -13485,10 +13465,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="c7b9d0d2-0928-4bc7-b1e7-d815d07dd502" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3b21ab7c-7e7a-493b-a43f-a219844d5b04">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5B9BAF98-50BE-4545-8DD0-8D32ADCB4CBD}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4D2A45D4-F0A1-4691-81DA-B2B59E7FD265}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="3b21ab7c-7e7a-493b-a43f-a219844d5b04"/>
+    <ds:schemaRef ds:uri="c7b9d0d2-0928-4bc7-b1e7-d815d07dd502"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -13505,20 +13516,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4D2A45D4-F0A1-4691-81DA-B2B59E7FD265}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5B9BAF98-50BE-4545-8DD0-8D32ADCB4CBD}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="3b21ab7c-7e7a-493b-a43f-a219844d5b04"/>
-    <ds:schemaRef ds:uri="c7b9d0d2-0928-4bc7-b1e7-d815d07dd502"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>